<commit_message>
Update MATLAB tool menu and add vehicle parameter automation
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/KPIs_Plots/eBus_KPIs_Plots_Bank.xlsx
+++ b/eBus_Functions/Post_Processing/KPIs_Plots/eBus_KPIs_Plots_Bank.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/65539596681e1364/Desktop/eBus_Simulation/eBus_Tool/eBus_Functions/Post_Processing/KPIs_Plots/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\KPIs_Plots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F661AFE4-D4DE-47AF-BC6B-7E1029E1BDD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF129B89-1401-4457-A155-22A17F0B41F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPIs" sheetId="1" r:id="rId1"/>
@@ -1866,7 +1866,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N505"/>
+  <dimension ref="A1:N504"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="2"/>
@@ -2607,6 +2607,30 @@
       <c r="N23" s="30"/>
     </row>
     <row r="24" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>21</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="29">
+        <v>1</v>
+      </c>
+      <c r="F24" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="H24" s="39" t="s">
+        <v>74</v>
+      </c>
       <c r="I24" s="39"/>
       <c r="J24" s="40"/>
       <c r="K24" s="40"/>
@@ -2616,13 +2640,13 @@
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C25" s="32" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D25" s="32" t="s">
         <v>47</v>
@@ -2631,13 +2655,13 @@
         <v>1</v>
       </c>
       <c r="F25" s="32" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G25" s="35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H25" s="39" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I25" s="39"/>
       <c r="J25" s="40"/>
@@ -2648,28 +2672,28 @@
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>22</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="C26" s="32" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="D26" s="32" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="E26" s="29">
         <v>1</v>
       </c>
       <c r="F26" s="32" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="G26" s="35" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="H26" s="39" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="I26" s="39"/>
       <c r="J26" s="40"/>
@@ -2680,13 +2704,13 @@
     </row>
     <row r="27" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>23</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>77</v>
+        <v>24</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>220</v>
       </c>
       <c r="C27" s="32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D27" s="32" t="s">
         <v>28</v>
@@ -2695,13 +2719,13 @@
         <v>1</v>
       </c>
       <c r="F27" s="32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G27" s="35" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H27" s="39" t="s">
-        <v>103</v>
+        <v>401</v>
       </c>
       <c r="I27" s="39"/>
       <c r="J27" s="40"/>
@@ -2712,13 +2736,13 @@
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C28" s="32" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="D28" s="32" t="s">
         <v>28</v>
@@ -2727,13 +2751,13 @@
         <v>1</v>
       </c>
       <c r="F28" s="32" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="G28" s="35" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H28" s="39" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="I28" s="39"/>
       <c r="J28" s="40"/>
@@ -2744,13 +2768,13 @@
     </row>
     <row r="29" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>221</v>
       </c>
       <c r="C29" s="32" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D29" s="32" t="s">
         <v>28</v>
@@ -2759,13 +2783,13 @@
         <v>1</v>
       </c>
       <c r="F29" s="32" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G29" s="35" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H29" s="39" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="I29" s="39"/>
       <c r="J29" s="40"/>
@@ -2776,28 +2800,28 @@
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>221</v>
       </c>
       <c r="C30" s="32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D30" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E30" s="29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G30" s="35" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H30" s="39" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="I30" s="39"/>
       <c r="J30" s="40"/>
@@ -2808,13 +2832,13 @@
     </row>
     <row r="31" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>221</v>
       </c>
       <c r="C31" s="32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D31" s="32" t="s">
         <v>28</v>
@@ -2823,13 +2847,13 @@
         <v>0</v>
       </c>
       <c r="F31" s="32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G31" s="35" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H31" s="39" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="I31" s="39"/>
       <c r="J31" s="40"/>
@@ -2840,28 +2864,28 @@
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>28</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>221</v>
+        <v>29</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>219</v>
       </c>
       <c r="C32" s="32" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="D32" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E32" s="29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" s="32" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="G32" s="35" t="s">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="H32" s="39" t="s">
-        <v>405</v>
+        <v>87</v>
       </c>
       <c r="I32" s="39"/>
       <c r="J32" s="40"/>
@@ -2872,13 +2896,13 @@
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>219</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="D33" s="32" t="s">
         <v>28</v>
@@ -2887,13 +2911,13 @@
         <v>1</v>
       </c>
       <c r="F33" s="32" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G33" s="35" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H33" s="39" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I33" s="39"/>
       <c r="J33" s="40"/>
@@ -2904,13 +2928,13 @@
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>219</v>
       </c>
       <c r="C34" s="32" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D34" s="32" t="s">
         <v>28</v>
@@ -2919,13 +2943,13 @@
         <v>1</v>
       </c>
       <c r="F34" s="32" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G34" s="35" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H34" s="39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I34" s="39"/>
       <c r="J34" s="40"/>
@@ -2936,13 +2960,13 @@
     </row>
     <row r="35" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>219</v>
       </c>
       <c r="C35" s="32" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D35" s="32" t="s">
         <v>28</v>
@@ -2951,13 +2975,13 @@
         <v>1</v>
       </c>
       <c r="F35" s="32" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G35" s="35" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H35" s="39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I35" s="39"/>
       <c r="J35" s="40"/>
@@ -2968,13 +2992,13 @@
     </row>
     <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>219</v>
       </c>
       <c r="C36" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D36" s="32" t="s">
         <v>28</v>
@@ -2983,13 +3007,13 @@
         <v>1</v>
       </c>
       <c r="F36" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G36" s="35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H36" s="39" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="I36" s="39"/>
       <c r="J36" s="40"/>
@@ -3000,28 +3024,26 @@
     </row>
     <row r="37" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>33</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>219</v>
+        <v>34</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>78</v>
       </c>
       <c r="C37" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="D37" s="32" t="s">
-        <v>28</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="D37" s="32"/>
       <c r="E37" s="29">
         <v>1</v>
       </c>
       <c r="F37" s="32" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="G37" s="35" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>87</v>
+        <v>137</v>
       </c>
       <c r="I37" s="39"/>
       <c r="J37" s="40"/>
@@ -3032,26 +3054,28 @@
     </row>
     <row r="38" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C38" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="D38" s="32"/>
+        <v>109</v>
+      </c>
+      <c r="D38" s="32" t="s">
+        <v>119</v>
+      </c>
       <c r="E38" s="29">
         <v>1</v>
       </c>
       <c r="F38" s="32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G38" s="35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H38" s="39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I38" s="39"/>
       <c r="J38" s="40"/>
@@ -3062,28 +3086,26 @@
     </row>
     <row r="39" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C39" s="32" t="s">
-        <v>109</v>
-      </c>
-      <c r="D39" s="32" t="s">
-        <v>119</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="D39" s="32"/>
       <c r="E39" s="29">
         <v>1</v>
       </c>
       <c r="F39" s="32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G39" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I39" s="39"/>
       <c r="J39" s="40"/>
@@ -3094,26 +3116,26 @@
     </row>
     <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C40" s="32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D40" s="32"/>
       <c r="E40" s="29">
         <v>1</v>
       </c>
       <c r="F40" s="32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G40" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H40" s="39" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I40" s="39"/>
       <c r="J40" s="40"/>
@@ -3124,26 +3146,26 @@
     </row>
     <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C41" s="32" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D41" s="32"/>
       <c r="E41" s="29">
         <v>1</v>
       </c>
       <c r="F41" s="32" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G41" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H41" s="39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I41" s="39"/>
       <c r="J41" s="40"/>
@@ -3154,26 +3176,26 @@
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C42" s="32" t="s">
-        <v>112</v>
+        <v>266</v>
       </c>
       <c r="D42" s="32"/>
       <c r="E42" s="29">
         <v>1</v>
       </c>
       <c r="F42" s="32" t="s">
-        <v>112</v>
+        <v>266</v>
       </c>
       <c r="G42" s="35" t="s">
-        <v>126</v>
+        <v>285</v>
       </c>
       <c r="H42" s="39" t="s">
-        <v>141</v>
+        <v>347</v>
       </c>
       <c r="I42" s="39"/>
       <c r="J42" s="40"/>
@@ -3184,26 +3206,26 @@
     </row>
     <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C43" s="32" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="D43" s="32"/>
       <c r="E43" s="29">
         <v>1</v>
       </c>
       <c r="F43" s="32" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="G43" s="35" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="H43" s="39" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="I43" s="39"/>
       <c r="J43" s="40"/>
@@ -3214,26 +3236,26 @@
     </row>
     <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C44" s="32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D44" s="32"/>
       <c r="E44" s="29">
         <v>1</v>
       </c>
       <c r="F44" s="32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G44" s="35" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H44" s="39" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="I44" s="39"/>
       <c r="J44" s="40"/>
@@ -3244,26 +3266,26 @@
     </row>
     <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C45" s="32" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D45" s="32"/>
       <c r="E45" s="29">
         <v>1</v>
       </c>
       <c r="F45" s="32" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G45" s="35" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H45" s="39" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="I45" s="39"/>
       <c r="J45" s="40"/>
@@ -3274,26 +3296,26 @@
     </row>
     <row r="46" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C46" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D46" s="32"/>
       <c r="E46" s="29">
         <v>1</v>
       </c>
       <c r="F46" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G46" s="35" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H46" s="39" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="I46" s="39"/>
       <c r="J46" s="40"/>
@@ -3304,26 +3326,26 @@
     </row>
     <row r="47" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C47" s="32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D47" s="32"/>
       <c r="E47" s="29">
         <v>1</v>
       </c>
       <c r="F47" s="32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G47" s="35" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H47" s="39" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="I47" s="39"/>
       <c r="J47" s="40"/>
@@ -3334,26 +3356,26 @@
     </row>
     <row r="48" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C48" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D48" s="32"/>
       <c r="E48" s="29">
         <v>1</v>
       </c>
       <c r="F48" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G48" s="35" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="H48" s="39" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="I48" s="39"/>
       <c r="J48" s="40"/>
@@ -3364,26 +3386,26 @@
     </row>
     <row r="49" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C49" s="32" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D49" s="32"/>
       <c r="E49" s="29">
         <v>1</v>
       </c>
       <c r="F49" s="32" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G49" s="35" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H49" s="39" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="I49" s="39"/>
       <c r="J49" s="40"/>
@@ -3394,26 +3416,26 @@
     </row>
     <row r="50" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C50" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D50" s="32"/>
       <c r="E50" s="29">
         <v>1</v>
       </c>
       <c r="F50" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G50" s="35" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H50" s="39" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="I50" s="39"/>
       <c r="J50" s="40"/>
@@ -3424,26 +3446,26 @@
     </row>
     <row r="51" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C51" s="32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D51" s="32"/>
       <c r="E51" s="29">
         <v>1</v>
       </c>
       <c r="F51" s="32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G51" s="35" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H51" s="39" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="I51" s="39"/>
       <c r="J51" s="40"/>
@@ -3454,26 +3476,26 @@
     </row>
     <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C52" s="32" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D52" s="32"/>
       <c r="E52" s="29">
         <v>1</v>
       </c>
       <c r="F52" s="32" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G52" s="35" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="H52" s="39" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I52" s="39"/>
       <c r="J52" s="40"/>
@@ -3484,26 +3506,26 @@
     </row>
     <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C53" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D53" s="32"/>
       <c r="E53" s="29">
         <v>1</v>
       </c>
       <c r="F53" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G53" s="35" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="H53" s="39" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I53" s="39"/>
       <c r="J53" s="40"/>
@@ -3514,26 +3536,26 @@
     </row>
     <row r="54" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C54" s="32" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D54" s="32"/>
       <c r="E54" s="29">
         <v>1</v>
       </c>
       <c r="F54" s="32" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G54" s="35" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H54" s="39" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="I54" s="39"/>
       <c r="J54" s="40"/>
@@ -3544,26 +3566,26 @@
     </row>
     <row r="55" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C55" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D55" s="32"/>
       <c r="E55" s="29">
         <v>1</v>
       </c>
       <c r="F55" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G55" s="35" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H55" s="39" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="I55" s="39"/>
       <c r="J55" s="40"/>
@@ -3574,26 +3596,26 @@
     </row>
     <row r="56" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C56" s="32" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D56" s="32"/>
       <c r="E56" s="29">
         <v>1</v>
       </c>
       <c r="F56" s="32" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G56" s="35" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H56" s="39" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="I56" s="39"/>
       <c r="J56" s="40"/>
@@ -3604,26 +3626,26 @@
     </row>
     <row r="57" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C57" s="32" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D57" s="32"/>
       <c r="E57" s="29">
         <v>1</v>
       </c>
       <c r="F57" s="32" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G57" s="35" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H57" s="39" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="I57" s="39"/>
       <c r="J57" s="40"/>
@@ -3634,26 +3656,26 @@
     </row>
     <row r="58" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C58" s="32" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D58" s="32"/>
       <c r="E58" s="29">
         <v>1</v>
       </c>
       <c r="F58" s="32" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G58" s="35" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H58" s="39" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="I58" s="39"/>
       <c r="J58" s="40"/>
@@ -3664,26 +3686,26 @@
     </row>
     <row r="59" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C59" s="32" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D59" s="32"/>
       <c r="E59" s="29">
         <v>1</v>
       </c>
       <c r="F59" s="32" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G59" s="35" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="H59" s="39" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I59" s="39"/>
       <c r="J59" s="40"/>
@@ -3694,26 +3716,26 @@
     </row>
     <row r="60" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C60" s="32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D60" s="32"/>
       <c r="E60" s="29">
         <v>1</v>
       </c>
       <c r="F60" s="32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G60" s="35" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H60" s="39" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I60" s="39"/>
       <c r="J60" s="40"/>
@@ -3724,26 +3746,26 @@
     </row>
     <row r="61" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C61" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D61" s="32"/>
       <c r="E61" s="29">
         <v>1</v>
       </c>
       <c r="F61" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G61" s="35" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H61" s="39" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I61" s="39"/>
       <c r="J61" s="40"/>
@@ -3754,26 +3776,26 @@
     </row>
     <row r="62" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C62" s="32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D62" s="32"/>
       <c r="E62" s="29">
         <v>1</v>
       </c>
       <c r="F62" s="32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G62" s="35" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H62" s="39" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="I62" s="39"/>
       <c r="J62" s="40"/>
@@ -3784,26 +3806,26 @@
     </row>
     <row r="63" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C63" s="32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D63" s="32"/>
       <c r="E63" s="29">
         <v>1</v>
       </c>
       <c r="F63" s="32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G63" s="35" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H63" s="39" t="s">
-        <v>327</v>
+        <v>375</v>
       </c>
       <c r="I63" s="39"/>
       <c r="J63" s="40"/>
@@ -3814,26 +3836,26 @@
     </row>
     <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C64" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D64" s="32"/>
       <c r="E64" s="29">
         <v>1</v>
       </c>
       <c r="F64" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G64" s="35" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H64" s="39" t="s">
-        <v>375</v>
+        <v>326</v>
       </c>
       <c r="I64" s="39"/>
       <c r="J64" s="40"/>
@@ -3844,26 +3866,26 @@
     </row>
     <row r="65" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C65" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D65" s="32"/>
       <c r="E65" s="29">
         <v>1</v>
       </c>
       <c r="F65" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G65" s="35" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H65" s="39" t="s">
-        <v>326</v>
+        <v>376</v>
       </c>
       <c r="I65" s="39"/>
       <c r="J65" s="40"/>
@@ -3874,26 +3896,26 @@
     </row>
     <row r="66" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C66" s="32" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D66" s="32"/>
       <c r="E66" s="29">
         <v>1</v>
       </c>
       <c r="F66" s="32" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G66" s="35" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="H66" s="39" t="s">
-        <v>376</v>
+        <v>325</v>
       </c>
       <c r="I66" s="39"/>
       <c r="J66" s="40"/>
@@ -3904,26 +3926,26 @@
     </row>
     <row r="67" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C67" s="32" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D67" s="32"/>
       <c r="E67" s="29">
         <v>1</v>
       </c>
       <c r="F67" s="32" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G67" s="35" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H67" s="39" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="I67" s="39"/>
       <c r="J67" s="40"/>
@@ -3934,26 +3956,26 @@
     </row>
     <row r="68" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C68" s="32" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D68" s="32"/>
       <c r="E68" s="29">
         <v>1</v>
       </c>
       <c r="F68" s="32" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G68" s="35" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H68" s="39" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="I68" s="39"/>
       <c r="J68" s="40"/>
@@ -3964,26 +3986,26 @@
     </row>
     <row r="69" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C69" s="32" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D69" s="32"/>
       <c r="E69" s="29">
         <v>1</v>
       </c>
       <c r="F69" s="32" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G69" s="35" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="H69" s="39" t="s">
-        <v>323</v>
+        <v>377</v>
       </c>
       <c r="I69" s="39"/>
       <c r="J69" s="40"/>
@@ -3994,26 +4016,26 @@
     </row>
     <row r="70" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C70" s="32" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D70" s="32"/>
       <c r="E70" s="29">
         <v>1</v>
       </c>
       <c r="F70" s="32" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G70" s="35" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="H70" s="39" t="s">
-        <v>377</v>
+        <v>322</v>
       </c>
       <c r="I70" s="39"/>
       <c r="J70" s="40"/>
@@ -4024,26 +4046,26 @@
     </row>
     <row r="71" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C71" s="32" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D71" s="32"/>
       <c r="E71" s="29">
         <v>1</v>
       </c>
       <c r="F71" s="32" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G71" s="35" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="H71" s="39" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="I71" s="39"/>
       <c r="J71" s="40"/>
@@ -4054,26 +4076,26 @@
     </row>
     <row r="72" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C72" s="32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D72" s="32"/>
       <c r="E72" s="29">
         <v>1</v>
       </c>
       <c r="F72" s="32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G72" s="35" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="H72" s="39" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I72" s="39"/>
       <c r="J72" s="40"/>
@@ -4084,26 +4106,26 @@
     </row>
     <row r="73" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C73" s="32" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D73" s="32"/>
       <c r="E73" s="29">
         <v>1</v>
       </c>
       <c r="F73" s="32" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G73" s="35" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="H73" s="39" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I73" s="39"/>
       <c r="J73" s="40"/>
@@ -4114,26 +4136,26 @@
     </row>
     <row r="74" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C74" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D74" s="32"/>
       <c r="E74" s="29">
         <v>1</v>
       </c>
       <c r="F74" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G74" s="35" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H74" s="39" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I74" s="39"/>
       <c r="J74" s="40"/>
@@ -4144,26 +4166,28 @@
     </row>
     <row r="75" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
-        <v>71</v>
-      </c>
-      <c r="B75" s="6" t="s">
-        <v>78</v>
+        <v>72</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="C75" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="D75" s="32"/>
+        <v>113</v>
+      </c>
+      <c r="D75" s="32" t="s">
+        <v>120</v>
+      </c>
       <c r="E75" s="29">
         <v>1</v>
       </c>
       <c r="F75" s="32" t="s">
-        <v>284</v>
+        <v>113</v>
       </c>
       <c r="G75" s="35" t="s">
-        <v>317</v>
+        <v>127</v>
       </c>
       <c r="H75" s="39" t="s">
-        <v>318</v>
+        <v>142</v>
       </c>
       <c r="I75" s="39"/>
       <c r="J75" s="40"/>
@@ -4174,28 +4198,28 @@
     </row>
     <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>79</v>
       </c>
       <c r="C76" s="32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D76" s="32" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E76" s="29">
         <v>1</v>
       </c>
       <c r="F76" s="32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G76" s="35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H76" s="39" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I76" s="39"/>
       <c r="J76" s="40"/>
@@ -4206,28 +4230,28 @@
     </row>
     <row r="77" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
-        <v>73</v>
-      </c>
-      <c r="B77" s="5" t="s">
-        <v>79</v>
+        <v>74</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>222</v>
       </c>
       <c r="C77" s="32" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D77" s="32" t="s">
-        <v>121</v>
+        <v>28</v>
       </c>
       <c r="E77" s="29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F77" s="32" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G77" s="35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H77" s="39" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I77" s="39"/>
       <c r="J77" s="40"/>
@@ -4238,28 +4262,28 @@
     </row>
     <row r="78" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
-        <v>74</v>
-      </c>
-      <c r="B78" s="6" t="s">
-        <v>222</v>
+        <v>75</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="C78" s="32" t="s">
-        <v>115</v>
+        <v>18</v>
       </c>
       <c r="D78" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E78" s="29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F78" s="32" t="s">
-        <v>115</v>
+        <v>18</v>
       </c>
       <c r="G78" s="35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H78" s="39" t="s">
-        <v>144</v>
+        <v>29</v>
       </c>
       <c r="I78" s="39"/>
       <c r="J78" s="40"/>
@@ -4270,13 +4294,13 @@
     </row>
     <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C79" s="32" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
       <c r="D79" s="32" t="s">
         <v>28</v>
@@ -4285,13 +4309,13 @@
         <v>1</v>
       </c>
       <c r="F79" s="32" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
       <c r="G79" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H79" s="39" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="I79" s="39"/>
       <c r="J79" s="40"/>
@@ -4302,13 +4326,13 @@
     </row>
     <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C80" s="32" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D80" s="32" t="s">
         <v>28</v>
@@ -4317,13 +4341,13 @@
         <v>1</v>
       </c>
       <c r="F80" s="32" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G80" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H80" s="39" t="s">
-        <v>58</v>
+        <v>145</v>
       </c>
       <c r="I80" s="39"/>
       <c r="J80" s="40"/>
@@ -4334,13 +4358,13 @@
     </row>
     <row r="81" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C81" s="32" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="D81" s="32" t="s">
         <v>28</v>
@@ -4349,13 +4373,13 @@
         <v>1</v>
       </c>
       <c r="F81" s="32" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="G81" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H81" s="39" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I81" s="39"/>
       <c r="J81" s="40"/>
@@ -4366,13 +4390,13 @@
     </row>
     <row r="82" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C82" s="32" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D82" s="32" t="s">
         <v>28</v>
@@ -4381,13 +4405,13 @@
         <v>1</v>
       </c>
       <c r="F82" s="32" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G82" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H82" s="39" t="s">
-        <v>146</v>
+        <v>84</v>
       </c>
       <c r="I82" s="39"/>
       <c r="J82" s="40"/>
@@ -4398,28 +4422,28 @@
     </row>
     <row r="83" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C83" s="32" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="D83" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E83" s="29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F83" s="32" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="G83" s="35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H83" s="39" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I83" s="39"/>
       <c r="J83" s="40"/>
@@ -4430,28 +4454,28 @@
     </row>
     <row r="84" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C84" s="32" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="D84" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E84" s="29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F84" s="32" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="G84" s="35" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H84" s="39" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I84" s="39"/>
       <c r="J84" s="40"/>
@@ -4462,13 +4486,13 @@
     </row>
     <row r="85" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
-        <v>81</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>230</v>
       </c>
       <c r="C85" s="32" t="s">
-        <v>94</v>
+        <v>231</v>
       </c>
       <c r="D85" s="32" t="s">
         <v>28</v>
@@ -4477,30 +4501,25 @@
         <v>1</v>
       </c>
       <c r="F85" s="32" t="s">
-        <v>94</v>
+        <v>231</v>
       </c>
       <c r="G85" s="35" t="s">
-        <v>136</v>
+        <v>236</v>
       </c>
       <c r="H85" s="39" t="s">
-        <v>86</v>
-      </c>
-      <c r="I85" s="39"/>
-      <c r="J85" s="40"/>
-      <c r="K85" s="40"/>
-      <c r="L85" s="40"/>
-      <c r="M85" s="37"/>
-      <c r="N85" s="30"/>
+        <v>145</v>
+      </c>
+      <c r="I85" s="41"/>
     </row>
     <row r="86" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C86" s="32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D86" s="32" t="s">
         <v>28</v>
@@ -4509,77 +4528,76 @@
         <v>1</v>
       </c>
       <c r="F86" s="32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G86" s="35" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H86" s="39" t="s">
-        <v>145</v>
-      </c>
-      <c r="I86" s="41"/>
+        <v>146</v>
+      </c>
     </row>
     <row r="87" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B87" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C87" s="32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D87" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E87" s="29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F87" s="32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G87" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H87" s="39" t="s">
-        <v>146</v>
+        <v>84</v>
       </c>
     </row>
     <row r="88" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B88" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C88" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D88" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E88" s="29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F88" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G88" s="35" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H88" s="39" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="89" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B89" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C89" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D89" s="32" t="s">
         <v>28</v>
@@ -4588,24 +4606,24 @@
         <v>1</v>
       </c>
       <c r="F89" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G89" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H89" s="39" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="90" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C90" s="32" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="D90" s="32" t="s">
         <v>28</v>
@@ -4617,21 +4635,24 @@
         <v>235</v>
       </c>
       <c r="G90" s="35" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="H90" s="39" t="s">
-        <v>86</v>
+        <v>243</v>
+      </c>
+      <c r="I90" s="42" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="91" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C91" s="32" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="D91" s="32" t="s">
         <v>28</v>
@@ -4643,24 +4664,28 @@
         <v>235</v>
       </c>
       <c r="G91" s="35" t="s">
-        <v>242</v>
-      </c>
-      <c r="H91" s="39" t="s">
-        <v>243</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="H91" s="39"/>
       <c r="I91" s="42" t="s">
-        <v>244</v>
+        <v>245</v>
+      </c>
+      <c r="J91" s="42" t="s">
+        <v>246</v>
+      </c>
+      <c r="K91" s="42" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="92" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>230</v>
       </c>
       <c r="C92" s="32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D92" s="32" t="s">
         <v>28</v>
@@ -4672,55 +4697,48 @@
         <v>235</v>
       </c>
       <c r="G92" s="35" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H92" s="39"/>
-      <c r="I92" s="42" t="s">
-        <v>245</v>
-      </c>
-      <c r="J92" s="42" t="s">
+      <c r="L92" s="42" t="s">
         <v>246</v>
-      </c>
-      <c r="K92" s="42" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="93" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
-        <v>89</v>
-      </c>
-      <c r="B93" s="6" t="s">
-        <v>230</v>
+        <v>90</v>
+      </c>
+      <c r="B93" s="5" t="s">
+        <v>348</v>
       </c>
       <c r="C93" s="32" t="s">
-        <v>251</v>
+        <v>349</v>
       </c>
       <c r="D93" s="32" t="s">
-        <v>28</v>
+        <v>360</v>
       </c>
       <c r="E93" s="29">
         <v>1</v>
       </c>
       <c r="F93" s="32" t="s">
-        <v>235</v>
+        <v>349</v>
       </c>
       <c r="G93" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="H93" s="39"/>
-      <c r="L93" s="42" t="s">
-        <v>246</v>
+        <v>363</v>
+      </c>
+      <c r="H93" s="39" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="94" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C94" s="32" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D94" s="32" t="s">
         <v>360</v>
@@ -4729,24 +4747,24 @@
         <v>1</v>
       </c>
       <c r="F94" s="32" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G94" s="35" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H94" s="39" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="95" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C95" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D95" s="32" t="s">
         <v>360</v>
@@ -4755,24 +4773,24 @@
         <v>1</v>
       </c>
       <c r="F95" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G95" s="35" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H95" s="39" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="96" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C96" s="32" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D96" s="32" t="s">
         <v>360</v>
@@ -4781,10 +4799,10 @@
         <v>1</v>
       </c>
       <c r="F96" s="32" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G96" s="35" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="H96" s="39" t="s">
         <v>408</v>
@@ -4792,13 +4810,13 @@
     </row>
     <row r="97" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C97" s="32" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D97" s="32" t="s">
         <v>360</v>
@@ -4807,74 +4825,72 @@
         <v>1</v>
       </c>
       <c r="F97" s="32" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G97" s="35" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="H97" s="39" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C98" s="32" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D98" s="32" t="s">
-        <v>360</v>
+        <v>206</v>
       </c>
       <c r="E98" s="29">
         <v>1</v>
       </c>
       <c r="F98" s="32" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G98" s="35" t="s">
-        <v>367</v>
-      </c>
-      <c r="H98" s="39" t="s">
-        <v>409</v>
-      </c>
+        <v>368</v>
+      </c>
+      <c r="H98" s="39"/>
     </row>
     <row r="99" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C99" s="32" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D99" s="32" t="s">
-        <v>206</v>
+        <v>47</v>
       </c>
       <c r="E99" s="29">
         <v>1</v>
       </c>
       <c r="F99" s="32" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G99" s="35" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H99" s="39"/>
     </row>
     <row r="100" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C100" s="32" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D100" s="32" t="s">
         <v>47</v>
@@ -4883,127 +4899,104 @@
         <v>1</v>
       </c>
       <c r="F100" s="32" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G100" s="35" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H100" s="39"/>
     </row>
     <row r="101" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C101" s="32" t="s">
-        <v>356</v>
-      </c>
-      <c r="D101" s="32" t="s">
-        <v>47</v>
-      </c>
+        <v>357</v>
+      </c>
+      <c r="D101" s="32"/>
       <c r="E101" s="29">
         <v>1</v>
       </c>
       <c r="F101" s="32" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G101" s="35" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="H101" s="39"/>
     </row>
     <row r="102" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C102" s="32" t="s">
-        <v>357</v>
-      </c>
-      <c r="D102" s="32"/>
+        <v>361</v>
+      </c>
+      <c r="D102" s="32" t="s">
+        <v>362</v>
+      </c>
       <c r="E102" s="29">
         <v>1</v>
       </c>
       <c r="F102" s="32" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="G102" s="35" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="H102" s="39"/>
     </row>
     <row r="103" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C103" s="32" t="s">
-        <v>361</v>
-      </c>
-      <c r="D103" s="32" t="s">
-        <v>362</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="D103" s="32"/>
       <c r="E103" s="29">
         <v>1</v>
       </c>
       <c r="F103" s="32" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="G103" s="35" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="H103" s="39"/>
     </row>
     <row r="104" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C104" s="32" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D104" s="32"/>
       <c r="E104" s="29">
         <v>1</v>
       </c>
       <c r="F104" s="32" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G104" s="35" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="H104" s="39"/>
     </row>
-    <row r="105" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="2">
-        <v>101</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="C105" s="32" t="s">
-        <v>359</v>
-      </c>
-      <c r="D105" s="32"/>
-      <c r="E105" s="29">
-        <v>1</v>
-      </c>
-      <c r="F105" s="32" t="s">
-        <v>359</v>
-      </c>
-      <c r="G105" s="35" t="s">
-        <v>374</v>
-      </c>
-      <c r="H105" s="39"/>
-    </row>
+    <row r="105" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="106" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="107" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="108" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -5403,10 +5396,9 @@
     <row r="502" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="503" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="504" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="505" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="G25:G113 G2:G23">
+  <conditionalFormatting sqref="G2:G112">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update DIVe batch processing and reorganize report templates
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/KPIs_Plots/eBus_KPIs_Plots_Bank.xlsx
+++ b/eBus_Functions/Post_Processing/KPIs_Plots/eBus_KPIs_Plots_Bank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\KPIs_Plots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF129B89-1401-4457-A155-22A17F0B41F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB15C2B-7ACA-46C0-895A-9865F8EBB33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPIs" sheetId="1" r:id="rId1"/>
@@ -2409,6 +2409,9 @@
       <c r="N16" s="30"/>
     </row>
     <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
       <c r="B17" s="6" t="s">
         <v>46</v>
       </c>
@@ -2429,7 +2432,7 @@
     </row>
     <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>46</v>
@@ -2460,6 +2463,9 @@
       <c r="N18" s="30"/>
     </row>
     <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
       <c r="B19" s="6" t="s">
         <v>46</v>
       </c>
@@ -2480,7 +2486,7 @@
     </row>
     <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>46</v>
@@ -2512,7 +2518,7 @@
     </row>
     <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>46</v>
@@ -2544,7 +2550,7 @@
     </row>
     <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>46</v>
@@ -2576,7 +2582,7 @@
     </row>
     <row r="23" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>46</v>
@@ -2608,7 +2614,7 @@
     </row>
     <row r="24" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>46</v>
@@ -2640,7 +2646,7 @@
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>46</v>
@@ -2672,7 +2678,7 @@
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>77</v>
@@ -2704,7 +2710,7 @@
     </row>
     <row r="27" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>220</v>
@@ -2736,7 +2742,7 @@
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>221</v>
@@ -2768,7 +2774,7 @@
     </row>
     <row r="29" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>221</v>
@@ -2800,7 +2806,7 @@
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>221</v>
@@ -2832,7 +2838,7 @@
     </row>
     <row r="31" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>221</v>
@@ -2864,7 +2870,7 @@
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>219</v>
@@ -2896,7 +2902,7 @@
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>219</v>
@@ -2928,7 +2934,7 @@
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>219</v>
@@ -2960,7 +2966,7 @@
     </row>
     <row r="35" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>219</v>
@@ -2992,7 +2998,7 @@
     </row>
     <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>219</v>
@@ -3024,7 +3030,7 @@
     </row>
     <row r="37" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>78</v>
@@ -3054,7 +3060,7 @@
     </row>
     <row r="38" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>78</v>
@@ -3086,7 +3092,7 @@
     </row>
     <row r="39" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>78</v>
@@ -3116,7 +3122,7 @@
     </row>
     <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>78</v>
@@ -3146,7 +3152,7 @@
     </row>
     <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>78</v>
@@ -3176,7 +3182,7 @@
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>78</v>
@@ -3206,7 +3212,7 @@
     </row>
     <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>78</v>
@@ -3236,7 +3242,7 @@
     </row>
     <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>78</v>
@@ -3266,7 +3272,7 @@
     </row>
     <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>78</v>
@@ -3296,7 +3302,7 @@
     </row>
     <row r="46" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>78</v>
@@ -3326,7 +3332,7 @@
     </row>
     <row r="47" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>78</v>
@@ -3356,7 +3362,7 @@
     </row>
     <row r="48" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>78</v>
@@ -3386,7 +3392,7 @@
     </row>
     <row r="49" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>78</v>
@@ -3416,7 +3422,7 @@
     </row>
     <row r="50" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>78</v>
@@ -3446,7 +3452,7 @@
     </row>
     <row r="51" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>78</v>
@@ -3476,7 +3482,7 @@
     </row>
     <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>78</v>
@@ -3506,7 +3512,7 @@
     </row>
     <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>78</v>
@@ -3536,7 +3542,7 @@
     </row>
     <row r="54" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>78</v>
@@ -3566,7 +3572,7 @@
     </row>
     <row r="55" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>78</v>
@@ -3596,7 +3602,7 @@
     </row>
     <row r="56" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>78</v>
@@ -3626,7 +3632,7 @@
     </row>
     <row r="57" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>78</v>
@@ -3656,7 +3662,7 @@
     </row>
     <row r="58" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>78</v>
@@ -3686,7 +3692,7 @@
     </row>
     <row r="59" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>78</v>
@@ -3716,7 +3722,7 @@
     </row>
     <row r="60" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>78</v>
@@ -3746,7 +3752,7 @@
     </row>
     <row r="61" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>78</v>
@@ -3776,7 +3782,7 @@
     </row>
     <row r="62" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>78</v>
@@ -3806,7 +3812,7 @@
     </row>
     <row r="63" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>78</v>
@@ -3836,7 +3842,7 @@
     </row>
     <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>78</v>
@@ -3866,7 +3872,7 @@
     </row>
     <row r="65" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>78</v>
@@ -3896,7 +3902,7 @@
     </row>
     <row r="66" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>78</v>
@@ -3926,7 +3932,7 @@
     </row>
     <row r="67" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>78</v>
@@ -3956,7 +3962,7 @@
     </row>
     <row r="68" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>78</v>
@@ -3986,7 +3992,7 @@
     </row>
     <row r="69" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>78</v>
@@ -4016,7 +4022,7 @@
     </row>
     <row r="70" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>78</v>
@@ -4046,7 +4052,7 @@
     </row>
     <row r="71" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>78</v>
@@ -4076,7 +4082,7 @@
     </row>
     <row r="72" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>78</v>
@@ -4106,7 +4112,7 @@
     </row>
     <row r="73" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>78</v>
@@ -4136,7 +4142,7 @@
     </row>
     <row r="74" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>78</v>
@@ -4166,7 +4172,7 @@
     </row>
     <row r="75" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>79</v>
@@ -4198,7 +4204,7 @@
     </row>
     <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>79</v>
@@ -4230,7 +4236,7 @@
     </row>
     <row r="77" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>222</v>
@@ -4262,7 +4268,7 @@
     </row>
     <row r="78" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>80</v>
@@ -4294,7 +4300,7 @@
     </row>
     <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>80</v>
@@ -4326,7 +4332,7 @@
     </row>
     <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>80</v>
@@ -4358,7 +4364,7 @@
     </row>
     <row r="81" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>80</v>
@@ -4390,7 +4396,7 @@
     </row>
     <row r="82" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>80</v>
@@ -4422,7 +4428,7 @@
     </row>
     <row r="83" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>80</v>
@@ -4454,7 +4460,7 @@
     </row>
     <row r="84" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>80</v>
@@ -4486,7 +4492,7 @@
     </row>
     <row r="85" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B85" s="6" t="s">
         <v>230</v>
@@ -4513,7 +4519,7 @@
     </row>
     <row r="86" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>230</v>
@@ -4539,7 +4545,7 @@
     </row>
     <row r="87" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B87" s="6" t="s">
         <v>230</v>
@@ -4565,7 +4571,7 @@
     </row>
     <row r="88" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B88" s="6" t="s">
         <v>230</v>
@@ -4591,7 +4597,7 @@
     </row>
     <row r="89" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B89" s="6" t="s">
         <v>230</v>
@@ -4617,7 +4623,7 @@
     </row>
     <row r="90" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>230</v>
@@ -4646,7 +4652,7 @@
     </row>
     <row r="91" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>230</v>
@@ -4679,7 +4685,7 @@
     </row>
     <row r="92" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>230</v>
@@ -4706,7 +4712,7 @@
     </row>
     <row r="93" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>348</v>
@@ -4732,7 +4738,7 @@
     </row>
     <row r="94" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>348</v>
@@ -4758,7 +4764,7 @@
     </row>
     <row r="95" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>348</v>
@@ -4784,7 +4790,7 @@
     </row>
     <row r="96" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>348</v>
@@ -4810,7 +4816,7 @@
     </row>
     <row r="97" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>348</v>
@@ -4836,7 +4842,7 @@
     </row>
     <row r="98" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>348</v>
@@ -4860,7 +4866,7 @@
     </row>
     <row r="99" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>348</v>
@@ -4884,7 +4890,7 @@
     </row>
     <row r="100" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>348</v>
@@ -4908,7 +4914,7 @@
     </row>
     <row r="101" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>348</v>
@@ -4930,7 +4936,7 @@
     </row>
     <row r="102" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>348</v>
@@ -4954,7 +4960,7 @@
     </row>
     <row r="103" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>348</v>
@@ -4976,7 +4982,7 @@
     </row>
     <row r="104" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>348</v>

</xml_diff>